<commit_message>
Last commit for the browser Metrics
</commit_message>
<xml_diff>
--- a/output/DashboardMetrics.xlsx
+++ b/output/DashboardMetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,6 +630,136 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>b1f6b192-1c11-4531-818f-1d88795d3168</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:18:44</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>HR Analytics Data Model</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;pbi_source=linkShare</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Page 1 - HR Analytics Data Model - Power BI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5/ReportSectiona3a61fc339266647faed?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>200</v>
+      </c>
+      <c r="H4" t="n">
+        <v>30.712</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="J4" t="n">
+        <v>10.014</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.321</v>
+      </c>
+      <c r="L4" t="n">
+        <v>41.714</v>
+      </c>
+      <c r="M4" t="n">
+        <v>120</v>
+      </c>
+      <c r="N4" t="n">
+        <v>115</v>
+      </c>
+      <c r="O4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fb85c077-64ba-40ed-9876-591c68adab5f</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:19:21</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sheet Cake Retail sales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/fc07298b-68d9-4b15-8dbd-92e6fbc11c3a/reports/18a733b5-a984-4763-b581-fe8a52ccb25a?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;pbi_source=linkShare</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1/4 Sheet Cake Retail Sales TY vs LY GCP - Power BI</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/fc07298b-68d9-4b15-8dbd-92e6fbc11c3a/reports/18a733b5-a984-4763-b581-fe8a52ccb25a/ReportSection2a28fc03c379139420ca?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>200</v>
+      </c>
+      <c r="H5" t="n">
+        <v>25.688</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J5" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="L5" t="n">
+        <v>36.589</v>
+      </c>
+      <c r="M5" t="n">
+        <v>132</v>
+      </c>
+      <c r="N5" t="n">
+        <v>125</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
made single main function run it with py -m automation.runner
</commit_message>
<xml_diff>
--- a/output/DashboardMetrics.xlsx
+++ b/output/DashboardMetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -760,6 +760,201 @@
         <v>4</v>
       </c>
       <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>8c3e4be8-88a2-466c-9ea6-eec93adb44be</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-02 22:20:07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HR Analytics Data Model</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;pbi_source=linkShare</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HR Analytics Data Model - Power BI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5/ReportSectiona3a61fc339266647faed?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>200</v>
+      </c>
+      <c r="H6" t="n">
+        <v>29.35</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="J6" t="n">
+        <v>10.017</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="L6" t="n">
+        <v>40.681</v>
+      </c>
+      <c r="M6" t="n">
+        <v>118</v>
+      </c>
+      <c r="N6" t="n">
+        <v>113</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>00476cc2-f74e-427a-9989-7fe724193b4c</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-02 22:28:08</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>HR Analytics Data Model</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;pbi_source=linkShare</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>HR Analytics Data Model - Power BI</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8bebcbe8-744a-42af-93f2-8ceec34939d5/ReportSectiona3a61fc339266647faed?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" t="n">
+        <v>23.392</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.631</v>
+      </c>
+      <c r="J7" t="n">
+        <v>10.042</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="L7" t="n">
+        <v>34.257</v>
+      </c>
+      <c r="M7" t="n">
+        <v>118</v>
+      </c>
+      <c r="N7" t="n">
+        <v>112</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4</v>
+      </c>
+      <c r="P7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10aeb5bf-f0e9-43e9-b3c9-c010683344b7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-02 22:29:28</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sheet Cake Retail sales</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/fc07298b-68d9-4b15-8dbd-92e6fbc11c3a/reports/18a733b5-a984-4763-b581-fe8a52ccb25a?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;pbi_source=linkShare</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1/4 Sheet Cake Retail Sales TY vs LY GCP - Power BI</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/fc07298b-68d9-4b15-8dbd-92e6fbc11c3a/reports/18a733b5-a984-4763-b581-fe8a52ccb25a/ReportSection2a28fc03c379139420ca?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>200</v>
+      </c>
+      <c r="H8" t="n">
+        <v>19.468</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10.015</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="L8" t="n">
+        <v>30.463</v>
+      </c>
+      <c r="M8" t="n">
+        <v>134</v>
+      </c>
+      <c r="N8" t="n">
+        <v>126</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
created the frontend folder
</commit_message>
<xml_diff>
--- a/output/DashboardMetrics.xlsx
+++ b/output/DashboardMetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1085,6 +1085,136 @@
         <v>4</v>
       </c>
       <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>19c04811-f06a-4d41-9a01-1c7b1013a6c0</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-08-03 20:01:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>HR Linkdin Learnings Trendence</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/5e460a68-6f15-41f3-a1fa-d7fbf7245850/reports/32bcac73-bf58-462e-9c8a-888f444f1f23/b336d82694c085080013?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi&amp;bookmarkGuid=5ac48e9e6d0a96011379</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HR Linkedin Learning GCP Prod - Power BI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/5e460a68-6f15-41f3-a1fa-d7fbf7245850/reports/32bcac73-bf58-462e-9c8a-888f444f1f23/b336d82694c085080013?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi&amp;bookmarkGuid=5ac48e9e6d0a96011379</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H11" t="n">
+        <v>39.442</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10.012</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="L11" t="n">
+        <v>50.154</v>
+      </c>
+      <c r="M11" t="n">
+        <v>154</v>
+      </c>
+      <c r="N11" t="n">
+        <v>150</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4</v>
+      </c>
+      <c r="P11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>64452df2-abce-4768-b176-90f8ec4e6413</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-03 20:02:21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>HR linkdin learningd</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/0718cb2f-ec2a-45ea-a57e-4cecce8bed5d/b336d82694c085080013?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>HR Linkedin Learning - Power BI</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/0718cb2f-ec2a-45ea-a57e-4cecce8bed5d/b336d82694c085080013?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>200</v>
+      </c>
+      <c r="H12" t="n">
+        <v>20.517</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="J12" t="n">
+        <v>10.007</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="L12" t="n">
+        <v>31.175</v>
+      </c>
+      <c r="M12" t="n">
+        <v>154</v>
+      </c>
+      <c r="N12" t="n">
+        <v>150</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Connected backend and frontend
</commit_message>
<xml_diff>
--- a/output/DashboardMetrics.xlsx
+++ b/output/DashboardMetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1215,6 +1215,136 @@
         <v>4</v>
       </c>
       <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08f31264-eb75-4cf3-bf1e-4600c0b279e2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-04 11:55:49</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dashboard A</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8e7017c6-9c78-46f5-b511-15b891ea7f2d/0a05895d0eb1d076c78b?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HR TA Report - Power BI</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/c1bacf56-2795-4173-8cee-dd7dba5c7e06/reports/8e7017c6-9c78-46f5-b511-15b891ea7f2d/0a05895d0eb1d076c78b?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>200</v>
+      </c>
+      <c r="H13" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="J13" t="n">
+        <v>10.003</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="L13" t="n">
+        <v>36.339</v>
+      </c>
+      <c r="M13" t="n">
+        <v>142</v>
+      </c>
+      <c r="N13" t="n">
+        <v>138</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>86616331-68cc-4391-9949-fe63eaba5a74</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-04 11:56:43</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dashboard B</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/5e460a68-6f15-41f3-a1fa-d7fbf7245850/reports/6af27fd3-971c-40e1-a8af-321942bf73a5/0a05895d0eb1d076c78b?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>HR TA Report GCP Prod - Power BI</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/groups/5e460a68-6f15-41f3-a1fa-d7fbf7245850/reports/6af27fd3-971c-40e1-a8af-321942bf73a5/0a05895d0eb1d076c78b?ctid=e7c6f609-f63a-4ec7-b71e-6734c4c9d231&amp;experience=power-bi</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>200</v>
+      </c>
+      <c r="H14" t="n">
+        <v>20.329</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="J14" t="n">
+        <v>10.009</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="L14" t="n">
+        <v>31.02</v>
+      </c>
+      <c r="M14" t="n">
+        <v>145</v>
+      </c>
+      <c r="N14" t="n">
+        <v>137</v>
+      </c>
+      <c r="O14" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>